<commit_message>
docs: conclui blocos B e D da ordem de execução e alinha preços de implantação
- ORDEM_EXECUCAO: itens 3, 7, 8 e 9 marcados
- ZELA_STATUS e CHANGELOG: Mapa de Habilidades validado nos 3 perfis
- Planilhas de preços com implantação de 600 a 1.200 (recalcular ao abrir no Excel)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SIMULACAO_PRECOS_ZELA.xlsx
+++ b/docs/SIMULACAO_PRECOS_ZELA.xlsx
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
     </row>
     <row r="18">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1500</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="19">

</xml_diff>